<commit_message>
Planilha v5 final: correções da revisão (Organograma, data em Cálculos, links C84/E84, premissas derivadas, textos)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014nxthFHMZF8aEXBVoEN5GT
</commit_message>
<xml_diff>
--- a/planilhas/Embracon_simulacao_tributaria_04.09.26_v5.xlsx
+++ b/planilhas/Embracon_simulacao_tributaria_04.09.26_v5.xlsx
@@ -2639,19 +2639,14 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>189699</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>149680</xdr:rowOff>
     </xdr:from>
-    <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>431745</xdr:colOff>
-      <xdr:row>35</xdr:row>
-      <xdr:rowOff>22772</xdr:rowOff>
-    </xdr:to>
+    <xdr:ext cx="14650773" cy="5045456"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="Imagem 1">
@@ -2682,20 +2677,15 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>96050</xdr:colOff>
       <xdr:row>35</xdr:row>
       <xdr:rowOff>54429</xdr:rowOff>
     </xdr:from>
-    <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>420574</xdr:colOff>
-      <xdr:row>64</xdr:row>
-      <xdr:rowOff>161895</xdr:rowOff>
-    </xdr:to>
+    <xdr:ext cx="14455142" cy="5630061"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="3" name="Imagem 2">
@@ -2726,7 +2716,7 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:twoCellAnchor>
+  </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
@@ -3358,8 +3348,9 @@
   <dimension ref="C2:E5"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
+    <col min="1" max="1" width="7.54296875" customWidth="1"/>
     <col min="3" max="3" width="16.453125" customWidth="1"/>
-    <col min="4" max="4" width="32" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -3413,7 +3404,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="26" customHeight="1">
+    <row r="5" ht="44" customHeight="1">
       <c r="C5" s="342" t="inlineStr">
         <is>
           <t xml:space="preserve">4 de setembro de 2026</t>
@@ -3436,7 +3427,7 @@
       <c r="J6" s="278"/>
       <c r="K6" s="278"/>
     </row>
-    <row r="8" ht="79.0" customHeight="1">
+    <row r="8" ht="64.0" customHeight="1">
       <c r="B8" s="284" t="inlineStr">
         <is>
           <t xml:space="preserve">O objetivo destes exemplos é ilustrar o impacto que a classificação da Transação como Combinação de Negócios (CPC 15) ou como Joint Operation (CPC 19) pode gerar no custo do investimento das Holdings e no caso de venda futura da participação remanescente de 60% da Embracon. Para isso, simulamos a venda com (i) preço inferior ao valor justo; (ii) preço idêntico ao valor justo; e (iii) preço superior ao valor justo — pela própria Holding ou pelas pessoas físicas (alíquota simplificada de 22,5% sobre o ganho de capital). Os números são meramente estimados e não devem ser utilizados para ilustrar custos e contingências reais. Todos os valores são vinculados às abas 'Premissas', 'Cálculos da Operação', 'CPC 19' e 'Alienação Futura (PJ x PF)'.</t>
@@ -3912,127 +3903,127 @@
       <c r="K24" s="278"/>
     </row>
     <row r="26" ht="19" customHeight="1">
-      <c r="B26" s="280" t="inlineStr">
+      <c r="C26" s="280" t="inlineStr">
         <is>
           <t xml:space="preserve">CPC 15 | Combinação de Negócios</t>
         </is>
       </c>
-      <c r="C26" s="280"/>
       <c r="D26" s="280"/>
-      <c r="F26" s="281" t="inlineStr">
+      <c r="E26" s="280"/>
+      <c r="G26" s="281" t="inlineStr">
         <is>
           <t xml:space="preserve">CPC 19 | Joint Operation</t>
         </is>
       </c>
-      <c r="G26" s="281"/>
       <c r="H26" s="281"/>
+      <c r="I26" s="281"/>
     </row>
     <row r="27" ht="30" customHeight="1">
-      <c r="B27" s="294" t="inlineStr">
+      <c r="C27" s="294" t="inlineStr">
         <is>
           <t xml:space="preserve">Preço</t>
         </is>
       </c>
-      <c r="C27" s="295" t="inlineStr">
+      <c r="D27" s="295" t="inlineStr">
         <is>
           <t xml:space="preserve">Venda pela PJ</t>
         </is>
       </c>
-      <c r="D27" s="295" t="inlineStr">
+      <c r="E27" s="295" t="inlineStr">
         <is>
           <t xml:space="preserve">Venda pela PF</t>
         </is>
       </c>
-      <c r="F27" s="294" t="inlineStr">
+      <c r="G27" s="294" t="inlineStr">
         <is>
           <t xml:space="preserve">Preço</t>
         </is>
       </c>
-      <c r="G27" s="295" t="inlineStr">
+      <c r="H27" s="295" t="inlineStr">
         <is>
           <t xml:space="preserve">Venda pela PJ</t>
         </is>
       </c>
-      <c r="H27" s="295" t="inlineStr">
+      <c r="I27" s="295" t="inlineStr">
         <is>
           <t xml:space="preserve">Venda pela PF</t>
         </is>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="B28" s="344">
+      <c r="C28" s="344">
         <f>'Alienação Futura (PJ x PF)'!C30</f>
         <v>1000</v>
       </c>
-      <c r="C28" s="309">
+      <c r="D28" s="309">
         <f>'Alienação Futura (PJ x PF)'!D30</f>
         <v>120.496</v>
       </c>
-      <c r="D28" s="309">
+      <c r="E28" s="309">
         <f>'Alienação Futura (PJ x PF)'!E30</f>
         <v>220.95</v>
       </c>
-      <c r="F28" s="344">
+      <c r="G28" s="344">
         <f>'Alienação Futura (PJ x PF)'!C30</f>
         <v>1000</v>
       </c>
-      <c r="G28" s="309">
+      <c r="H28" s="309">
         <f>'Alienação Futura (PJ x PF)'!F30</f>
         <v>999.804</v>
       </c>
-      <c r="H28" s="309">
+      <c r="I28" s="309">
         <f>'Alienação Futura (PJ x PF)'!G30</f>
         <v>999.804</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="B29" s="344">
+      <c r="C29" s="344">
         <f>'Alienação Futura (PJ x PF)'!C31</f>
         <v>3573</v>
       </c>
-      <c r="C29" s="309">
+      <c r="D29" s="309">
         <f>'Alienação Futura (PJ x PF)'!D31</f>
         <v>995.316</v>
       </c>
-      <c r="D29" s="309">
+      <c r="E29" s="309">
         <f>'Alienação Futura (PJ x PF)'!E31</f>
         <v>799.875</v>
       </c>
-      <c r="F29" s="344">
+      <c r="G29" s="344">
         <f>'Alienação Futura (PJ x PF)'!C31</f>
         <v>3573</v>
       </c>
-      <c r="G29" s="309">
+      <c r="H29" s="309">
         <f>'Alienação Futura (PJ x PF)'!F31</f>
         <v>999.804</v>
       </c>
-      <c r="H29" s="309">
+      <c r="I29" s="309">
         <f>'Alienação Futura (PJ x PF)'!G31</f>
         <v>999.804</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="B30" s="344">
+      <c r="C30" s="344">
         <f>'Alienação Futura (PJ x PF)'!C32</f>
         <v>5000</v>
       </c>
-      <c r="C30" s="309">
+      <c r="D30" s="309">
         <f>'Alienação Futura (PJ x PF)'!D32</f>
         <v>1480.496</v>
       </c>
-      <c r="D30" s="309">
+      <c r="E30" s="309">
         <f>'Alienação Futura (PJ x PF)'!E32</f>
         <v>1120.95</v>
       </c>
-      <c r="F30" s="344">
+      <c r="G30" s="344">
         <f>'Alienação Futura (PJ x PF)'!C32</f>
         <v>5000</v>
       </c>
-      <c r="G30" s="309">
+      <c r="H30" s="309">
         <f>'Alienação Futura (PJ x PF)'!F32</f>
         <v>1484.984</v>
       </c>
-      <c r="H30" s="309">
+      <c r="I30" s="309">
         <f>'Alienação Futura (PJ x PF)'!G32</f>
         <v>1320.879</v>
       </c>
@@ -4088,7 +4079,7 @@
     <row r="36" ht="49.0" customHeight="1">
       <c r="B36" s="285" t="inlineStr">
         <is>
-          <t xml:space="preserve">• CPC 19 elimina a discussão sobre o custo, mas ao preço de reconhecer ganho de AVJ sobre toda a JO — inclusive a Embracon, que no CPC 15 não é reavaliada — com IRPJ/CSLL de 34% carimbado e devido na venda em qualquer cenário de preço, sem a alternativa da PF. Além disso, o valor patrimonial das Holdings sobe ao valor justo, com impacto direto na base de cálculo do ITCMD (tema não tratado neste material).</t>
+          <t xml:space="preserve">• CPC 19 elimina a discussão sobre o custo, mas ao preço de reconhecer ganho de AVJ sobre toda a JO — inclusive a Embracon, que no CPC 15 não é reavaliada — com IRPJ/CSLL de 34% carimbado e devido na venda em qualquer cenário de preço, sem a alternativa da PF. Além disso, o valor patrimonial das Holdings poderá subir ao valor justo (reconhecimento da CNP e da Embracon), com possível repercussão na base de cálculo do ITCMD, a depender do critério legal aplicável (tema não analisado neste material).</t>
         </is>
       </c>
       <c r="C36" s="285"/>
@@ -4117,7 +4108,7 @@
       <c r="J37" s="285"/>
       <c r="K37" s="285"/>
     </row>
-    <row r="38" ht="49.0" customHeight="1">
+    <row r="38" ht="34.0" customHeight="1">
       <c r="B38" s="284" t="inlineStr">
         <is>
           <t xml:space="preserve">Ressalvas: valores ilustrativos em R$ milhões, data-base 30.06.2026, com as premissas da aba 'Premissas'. As Holdings estão no lucro presumido; na venda futura, a carga efetiva na PJ poderia ser reduzida com a opção pelo lucro real e a existência de prejuízos compensáveis. O custo das quotas nas PFs é premissa ilustrativa a confirmar. O material não avalia o ITCMD.</t>
@@ -4149,8 +4140,8 @@
     <mergeCell ref="F21:K21"/>
     <mergeCell ref="F22:K22"/>
     <mergeCell ref="B24:K24"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="F26:H26"/>
+    <mergeCell ref="C26:E26"/>
+    <mergeCell ref="G26:I26"/>
     <mergeCell ref="B31:K31"/>
     <mergeCell ref="B33:K33"/>
     <mergeCell ref="B35:K35"/>
@@ -4187,8 +4178,12 @@
         <v>276</v>
       </c>
     </row>
-    <row r="5" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="E5" s="102"/>
+    <row r="5" spans="2:11" ht="26" customHeight="1">
+      <c r="E5" s="342" t="inlineStr">
+        <is>
+          <t>4 de setembro de 2026</t>
+        </is>
+      </c>
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.35">
       <c r="C9" s="105"/>
@@ -4995,10 +4990,12 @@
         <v>148</v>
       </c>
       <c r="C84" s="188">
+        <f>D69</f>
         <v>600</v>
       </c>
       <c r="D84" s="188"/>
       <c r="E84" s="188">
+        <f>D70</f>
         <v>600</v>
       </c>
       <c r="F84" s="188"/>
@@ -5320,7 +5317,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="26" customHeight="1">
+    <row r="5" ht="44" customHeight="1">
       <c r="C5" s="342" t="inlineStr">
         <is>
           <t xml:space="preserve">4 de setembro de 2026</t>
@@ -5705,7 +5702,7 @@
       <c r="J24" s="278"/>
       <c r="K24" s="278"/>
     </row>
-    <row r="26" ht="79.0" customHeight="1">
+    <row r="26" ht="64.0" customHeight="1">
       <c r="B26" s="284" t="inlineStr">
         <is>
           <t xml:space="preserve">Simulamos a venda dos 60% remanescentes em três preços — abaixo, igual e acima do valor justo (60% do valor justo da JO). No CPC 15, o imposto incide sobre a diferença entre o preço e o custo fiscal incrementado remanescente (aba 'Cálculos da Operação'). No CPC 19, o imposto diferido de 34% sobre o AVJ é devido de qualquer forma e funciona como piso; se o preço superar o valor justo, o excedente também é tributado. Na venda pelas pessoas físicas (após 'subir' as ações das Holdings para as PFs), aplica-se a alíquota simplificada de 22,5% sobre o ganho; porém o custo das PFs é o custo das quotas das Holdings, muito inferior ao custo da Holding, e no CPC 19 o imposto carimbado permanece na Holding mesmo que a venda seja feita pela PF.</t>
@@ -5910,7 +5907,7 @@
       <c r="J33" s="286"/>
       <c r="K33" s="286"/>
     </row>
-    <row r="34" ht="64.0" customHeight="1">
+    <row r="34" ht="49.0" customHeight="1">
       <c r="B34" s="284" t="inlineStr">
         <is>
           <t xml:space="preserve">Leitura: em preços iguais ou superiores ao valor justo, a diferença entre os regimes na venda pela Holding é pequena e corresponde a 34% da mais-valia da CNP — a única camada que o CPC 15 leva ao custo e o CPC 19 tributa. Abaixo do valor justo, o CPC 19 é substancialmente mais oneroso, porque o imposto diferido não diminui com o preço. A venda pela PF só é vantajosa no CPC 15, e apenas a partir de preços em que a alíquota menor compensa o custo menor das quotas; no CPC 19 ela não elimina o imposto carimbado, que permanece na Holding.</t>
@@ -6302,7 +6299,7 @@
         <v>159.392631090487</v>
       </c>
     </row>
-    <row r="54" ht="64.0" customHeight="1">
+    <row r="54" ht="49.0" customHeight="1">
       <c r="B54" s="284" t="inlineStr">
         <is>
           <t xml:space="preserve">Leitura: cada degrau de risco tem valor fixo, igual a 34% da camada negada, independentemente do preço. O RISCO 2 coincide com o CPC 19 nas vendas ao valor justo ou acima (mesma base contábil); abaixo do valor justo o CPC 19 continua pior, pelo piso do imposto carimbado. O RISCO 1 supera o CPC 19 em qualquer preço a partir do valor justo: se a tese de neutralidade do reflexo do PL contábil da CNP fosse integralmente afastada, o CPC 15 deixaria de ser o cenário mais favorável na venda futura — daí a importância de documentar a tese e o laudo de avaliação (PPA).</t>
@@ -7965,7 +7962,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="26" customHeight="1">
+    <row r="5" ht="44" customHeight="1">
       <c r="C5" s="342" t="inlineStr">
         <is>
           <t xml:space="preserve">4 de setembro de 2026</t>
@@ -7975,7 +7972,7 @@
     <row r="6" ht="18.5" customHeight="1">
       <c r="B6" s="278" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fatos da operação (Acordo de Investimento e material SF de 31.08.2026)</t>
+          <t xml:space="preserve">Fatos da operação (Acordo de Investimento, Ofício BACEN 31070/2026, calls Deloitte/SF e material SF de 31.08.2026)</t>
         </is>
       </c>
       <c r="C6" s="278"/>
@@ -8166,18 +8163,19 @@
       <c r="J19" s="286"/>
       <c r="K19" s="286"/>
     </row>
-    <row r="20" ht="15" customHeight="1">
-      <c r="B20" s="329" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Investimento original — Savian (50%)</t>
-        </is>
-      </c>
-      <c r="C20" s="330">
+    <row r="20" ht="30" customHeight="1">
+      <c r="B20" s="286" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Investimento original — Savian (50% do PL da Embracon)</t>
+        </is>
+      </c>
+      <c r="C20" s="302">
+        <f>C19/2</f>
         <v>127</v>
       </c>
       <c r="D20" s="286" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custo histórico das ações da Embracon na Savian</t>
+          <t xml:space="preserve">Derivado: as Holdings são simétricas no modelo (50/50); a aba 'Cálculos da Operação' dobra a coluna Savian para obter os totais</t>
         </is>
       </c>
       <c r="E20" s="286"/>
@@ -8188,18 +8186,19 @@
       <c r="J20" s="286"/>
       <c r="K20" s="286"/>
     </row>
-    <row r="21" ht="15" customHeight="1">
-      <c r="B21" s="329" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Investimento original — JVFJ (50%)</t>
-        </is>
-      </c>
-      <c r="C21" s="330">
+    <row r="21" ht="30" customHeight="1">
+      <c r="B21" s="286" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Investimento original — JVFJ (50% do PL da Embracon)</t>
+        </is>
+      </c>
+      <c r="C21" s="302">
+        <f>C20</f>
         <v>127</v>
       </c>
       <c r="D21" s="286" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custo histórico das ações da Embracon na JVFJ</t>
+          <t xml:space="preserve">Derivado: igual ao custo da Savian (simetria das Holdings)</t>
         </is>
       </c>
       <c r="E21" s="286"/>
@@ -8542,7 +8541,7 @@
     <row r="41" ht="18.5" customHeight="1">
       <c r="B41" s="278" t="inlineStr">
         <is>
-          <t xml:space="preserve">Premissas fiscais e ressalvas (material SF de 31.08.2026)</t>
+          <t xml:space="preserve">Premissas fiscais e ressalvas (material SF de 31.08.2026 e critérios adotados neste modelo)</t>
         </is>
       </c>
       <c r="C41" s="278"/>
@@ -8555,10 +8554,10 @@
       <c r="J41" s="278"/>
       <c r="K41" s="278"/>
     </row>
-    <row r="43" ht="34.0" customHeight="1">
+    <row r="43" ht="49.0" customHeight="1">
       <c r="B43" s="285" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Custo alocado no cash-out: a secundária é tratada como concomitante à incorporação e o custo de cada Holding é alocado proporcionalmente à fração alienada (13,1% ÷ 43,1%). O imposto do cash-out é apurado na aba 'Cálculos da Operação' nos cenários A (custo original) e B (custo incrementado).</t>
+          <t xml:space="preserve">• Custo alocado no cash-out (critério deste modelo, herdado da aba 'Cálculos da Operação'; o material SF de 31.08 alocava 26,2% do custo, 13,1% de cada Holding): a secundária é tratada como concomitante à incorporação e o custo de cada Holding é alocado proporcionalmente à fração alienada (13,1% ÷ 43,1%). O imposto do cash-out é apurado na aba 'Cálculos da Operação' nos cenários A (custo original) e B (custo incrementado).</t>
         </is>
       </c>
       <c r="C43" s="285"/>
@@ -8571,7 +8570,7 @@
       <c r="J43" s="285"/>
       <c r="K43" s="285"/>
     </row>
-    <row r="44" ht="49.0" customHeight="1">
+    <row r="44" ht="34.0" customHeight="1">
       <c r="B44" s="285" t="inlineStr">
         <is>
           <t xml:space="preserve">• Regime das Holdings: lucro presumido — premissa relevante para a tributação do cash-out. Na futura alienação dos 60% remanescentes, a carga poderá ser reduzida se, à época, as Holdings estiverem no lucro real e dispuserem de prejuízos fiscais e bases negativas de CSLL compensáveis, observadas as limitações aplicáveis.</t>
@@ -8590,7 +8589,7 @@
     <row r="45" ht="49.0" customHeight="1">
       <c r="B45" s="285" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Segregação de risco no CPC 15: o custo das Holdings é aberto em custo original (incontroverso), reflexo do PL contábil da CNP (neutralidade do MEP — art. 33, §2º, do DL 1.598/77; precedente WTorre, com decisões CARF de 2024 em sentido contrário) e reflexo da mais-valia (parcela mais exposta). No material de 31.08 a mais-valia era estimada em 34,6% do PL da CNP (proporção DTT 300/866); aqui é o valor de mercado menos o PL contábil.</t>
+          <t xml:space="preserve">• Segregação de risco no CPC 15: o custo das Holdings é aberto em custo original (incontroverso), reflexo do PL contábil da CNP (neutralidade do MEP — art. 33, §2º, do DL 1.598/77; precedente WTorre, com decisões CARF de 2024 em sentido contrário — fundamentos discutidos nas calls com a SF) e reflexo da mais-valia (parcela mais exposta). No material de 31.08 a mais-valia era estimada em 34,6% do PL da CNP (proporção DTT 300/866); aqui é o valor de mercado menos o PL contábil.</t>
         </is>
       </c>
       <c r="C45" s="285"/>
@@ -8721,7 +8720,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="26" customHeight="1">
+    <row r="5" ht="44" customHeight="1">
       <c r="C5" s="342" t="inlineStr">
         <is>
           <t xml:space="preserve">4 de setembro de 2026</t>
@@ -8744,7 +8743,7 @@
       <c r="J6" s="278"/>
       <c r="K6" s="278"/>
     </row>
-    <row r="8" ht="94.0" customHeight="1">
+    <row r="8" ht="79.0" customHeight="1">
       <c r="B8" s="284" t="inlineStr">
         <is>
           <t xml:space="preserve">Na operação em conjunto (CPC 19), leitura sustentada pela Deloitte a partir dos vetos qualificados da CNP, as Holdings deixam de avaliar o investimento pelo método de equivalência patrimonial e passam a reconhecer diretamente a sua parcela (60%) dos ativos e passivos da JO — Embracon e CNP — a valor justo. Isso inclui o valor justo da própria Embracon, que no CPC 15 não é reavaliada. O ganho de avaliação a valor justo (AVJ) não é tributado no reconhecimento, desde que controlado em subconta (arts. 13 e 14 da Lei 12.973/14), mas fica 'carimbado': o IRPJ/CSLL de 34% sobre o AVJ é devido quando o investimento for realizado (venda), qualquer que seja o preço e independentemente de quem venda. As premissas (valor justo da Embracon pelo EV do Acordo de Investimento e valor de mercado da CNP) vêm da aba 'Premissas'.</t>
@@ -9443,7 +9442,7 @@
       <c r="J41" s="293"/>
       <c r="K41" s="293"/>
     </row>
-    <row r="43" ht="64.0" customHeight="1">
+    <row r="43" ht="49.0" customHeight="1">
       <c r="B43" s="284" t="inlineStr">
         <is>
           <t xml:space="preserve">Leitura: no CPC 19 o custo das Holdings sobe para 60% do valor justo de toda a JO, mas o acréscimo é integralmente 'carimbado' — o IR diferido de 34% sobre o AVJ é devido na venda, qualquer que seja o preço, e permanece na Holding mesmo que a venda seja feita pelas pessoas físicas. Elimina-se a discussão sobre o custo, ao preço de reconhecer ganho sobre a própria Embracon (não reavaliada no CPC 15) e de elevar o valor patrimonial das Holdings, com possível impacto na base do ITCMD. A comparação com o CPC 15 na venda futura está na aba 'Alienação Futura (PJ x PF)'.</t>

</xml_diff>